<commit_message>
practica 2 acabada ac1
</commit_message>
<xml_diff>
--- a/AC1/Practica1/Auditoria_EncuestaCOVID_40.xlsx
+++ b/AC1/Practica1/Auditoria_EncuestaCOVID_40.xlsx
@@ -4017,7 +4017,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>bebidas_1</t>
+          <t>bebidas_1_clean</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>bebidas_1</t>
+          <t>bebidas_2_clean</t>
         </is>
       </c>
     </row>
@@ -4139,7 +4139,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>bebidas_1</t>
+          <t>bebidas_3_clean</t>
         </is>
       </c>
     </row>
@@ -4200,7 +4200,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>bebidas_1</t>
+          <t>bebidas_4_clean</t>
         </is>
       </c>
     </row>

</xml_diff>